<commit_message>
suricat testet funker i CML og oppdatet scripts
</commit_message>
<xml_diff>
--- a/NO_MPLS_SAD/demo_no_mpls.xlsx
+++ b/NO_MPLS_SAD/demo_no_mpls.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\NO_MPLS_SAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D57BF4F-8D10-450D-B670-CDBF6187C342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64F6F03-3C24-48D5-AAD3-1CE8B27A124A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28440" yWindow="0" windowWidth="23265" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site 1 (HUB)" sheetId="1" r:id="rId1"/>
     <sheet name="Site 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Site 3" sheetId="4" r:id="rId3"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -57,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="64">
   <si>
     <t>site</t>
   </si>
@@ -209,9 +211,6 @@
     <t>span_mode</t>
   </si>
   <si>
-    <t>ERSPAN</t>
-  </si>
-  <si>
     <t>SW</t>
   </si>
   <si>
@@ -236,9 +235,6 @@
     <t>num_port_ledig</t>
   </si>
   <si>
-    <t>10.1-200.1-20.5-30.5-40.2</t>
-  </si>
-  <si>
     <t>erspan_destination</t>
   </si>
   <si>
@@ -252,13 +248,16 @@
   </si>
   <si>
     <t>10.51.0.10</t>
+  </si>
+  <si>
+    <t>SPAN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -313,16 +312,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
@@ -357,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -392,36 +381,49 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="111">
+  <dxfs count="69">
     <dxf>
       <font>
         <color theme="1"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -431,22 +433,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -456,343 +443,39 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
         <sz val="11"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
         <sz val="11"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -966,73 +649,6 @@
         <color rgb="FF000000"/>
         <name val="Arial"/>
         <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
       </font>
     </dxf>
     <dxf>
@@ -1349,6 +965,27 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Site 1 (HUB)"/>
+      <sheetName val="Site 2"/>
+      <sheetName val="Site 3"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:J2">
   <tableColumns count="10">
@@ -1358,10 +995,10 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="67"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="66"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="dns_servers" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="dns_servers" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1370,26 +1007,26 @@
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell161824282532" displayName="Tabell161824282532" ref="A28:L29" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="SW" dataDxfId="80">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="SW" dataDxfId="10">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="MGMT Vlan" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="MGMT ip" dataDxfId="78">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="MGMT Vlan" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="MGMT ip" dataDxfId="8">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="gateway" dataDxfId="77">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="gateway" dataDxfId="7">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="mask" dataDxfId="76">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="mask" dataDxfId="6">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="num_ports_tot" dataDxfId="75"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="skiped_ports" dataDxfId="74"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="num_downlink" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="vlan-antall" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="intf_prefix" dataDxfId="71"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="num_port_ledig" dataDxfId="70">
-      <calculatedColumnFormula>IF($A29=1,F29-G29-H29*$F$26-2,F29-G29-(1+H29)*$F$26-1)</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="num_ports_tot" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="skiped_ports" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="num_downlink" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="vlan-antall" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="intf_prefix" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="num_port_ledig" dataDxfId="0">
+      <calculatedColumnFormula array="1">[1]!Tabell161824282532[num_port_ledig]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{5BF5BD4F-225D-489A-8CDF-AAA6E48E5D60}" name="MONITORING ip">
       <calculatedColumnFormula>LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</calculatedColumnFormula>
@@ -1416,7 +1053,7 @@
       <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{3FDE25A7-0BCB-41BA-9E6B-B97A44D97EF9}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{4F21A854-19B3-4F08-8736-4A49F53BB969}" name="antall-res" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{4F21A854-19B3-4F08-8736-4A49F53BB969}" name="antall-res" dataDxfId="38"/>
     <tableColumn id="10" xr3:uid="{EB637840-6D35-4793-BE43-FF44BBC60DCE}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{99B9B3BB-6A06-4A9B-B262-495BFC762025}" name="pri-1-10"/>
   </tableColumns>
@@ -1437,137 +1074,6 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{29423377-EE71-45EC-AE04-512C3676B300}" name="Tabell18" displayName="Tabell18" ref="A1:I2" dataDxfId="41">
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C426CE2C-D824-495E-9943-0D5ED22178FC}" name="site" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{BD14A14C-CA02-4292-9A53-DBBFAEFFB41E}" name="intf_prefix" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{1E884DEF-6FA0-43D2-90D1-A472ED2D772F}" name="router-id" dataDxfId="38">
-      <calculatedColumnFormula>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{5C62684E-F01D-41F8-91C7-33CAC2305C15}" name="brukernavn" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{270B3B2A-8408-4EDF-B211-8DE1F1AB0681}" name="passord" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{9804D10C-4308-4EBD-A637-0ED093054024}" name="vty_lines" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{B0910EE6-E1E3-4DBC-9F9C-47058BA9B153}" name="secret" dataDxfId="34"/>
-    <tableColumn id="8" xr3:uid="{D19E2A7E-21D0-4E2A-88C9-9F37D9A65437}" name="tacacs_key" dataDxfId="33">
-      <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="9" xr3:uid="{068D3A60-B781-41C3-BF0A-B042AD809343}" name="dns_servers" dataDxfId="32"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E6493EE3-7235-424D-A185-8FB87B73E9D5}" name="Tabell49" displayName="Tabell49" ref="A18:J23" dataDxfId="31">
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{14E90C76-B5F6-4A0B-A8EA-BBD1846F7ADE}" name="tunnel id" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{1DD92107-ED9E-41DA-9538-710D3656664D}" name="vrf" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{9CD976E2-E62F-4E14-BA9A-80672F5BC615}" name="ip address" dataDxfId="28">
-      <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{D92BBF85-664B-4383-9EDD-4C7538D00C07}" name="mask" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{41200B4B-99C3-46CD-8919-D19A650DFC09}" name="source" dataDxfId="26">
-      <calculatedColumnFormula>$C$2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{181D5214-8751-4D00-98A5-040FCE4E5826}" name="destination" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{595FE496-14D9-4619-8CC2-BDE4B0AE5AE1}" name="gre mode" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{C91D47FC-885E-4808-80A0-244D7156BD13}" name="network-id" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{D7BBBCE6-3579-420D-920C-EF19B478A7C2}" name="ipsec" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{E379820A-7358-40BE-83E4-07100824C704}" name="ipsec key" dataDxfId="21"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{7318DFAD-8A4D-4CFA-8FA6-6B5A78470C24}" name="Tabell1319253010" displayName="Tabell1319253010" ref="A25:H26" dataDxfId="20">
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{F6D980DA-8008-4018-B306-D36AE654DA5F}" name="site" dataDxfId="19">
-      <calculatedColumnFormula>A2</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{0D82B2DE-B4FA-4290-8C52-0CD4C0EAA67D}" name="brukernavn" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{27B9EF4E-512F-4DAC-8CB6-D2912CB2CDDA}" name="passord" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{6414CFB9-90E9-4655-838B-2676C80D7C06}" name="vty_lines" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{D51FD26F-2705-47EA-AED0-D3C21699B51F}" name="secret" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{ABC2D354-96CD-4993-8E5C-3CCEFAEF4846}" name="etherchan_num" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{3F9B25BE-C31E-4660-A97F-1B6AF14759A6}" name="span_mode" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{CA2E1FD4-EBFB-4BF5-8DD2-EE090C2F889B}" name="erspan_destination" dataDxfId="12"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{8BA68FF7-7C6C-4673-9B18-11015BB5ECE9}" name="Tabell16182428253212" displayName="Tabell16182428253212" ref="A28:L29" totalsRowShown="0">
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{8ADEAF6D-0562-4F81-93E4-69481AB6E718}" name="SW" dataDxfId="11">
-      <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{795F6504-A97F-4DFB-87AB-D0C3A93E475F}" name="MGMT Vlan" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{074C8822-FEF3-4C00-8C20-E4AAA6F87C8F}" name="MGMT ip" dataDxfId="9">
-      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A29)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{9E7BBCA3-A734-4692-A8F8-31365B75A063}" name="gateway" dataDxfId="8">
-      <calculatedColumnFormula>$E$5</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="5" xr3:uid="{B9D0B580-B85A-45C6-8EE9-922E6A0BDCD5}" name="mask" dataDxfId="7">
-      <calculatedColumnFormula>$F$5</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{136103A4-087C-4FA7-8332-FE71D232375E}" name="num_ports_tot" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{A0C44AB8-80BB-4052-A5FD-EE8530AB6772}" name="skiped_ports" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{52404E39-8CD5-4B37-A91F-C35409540738}" name="num_downlink" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{5B37CE82-3036-45D8-A546-50FF289EDBAD}" name="vlan-antall" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{79F10BE9-3D80-4FF6-A4B6-9184B24A72B4}" name="intf_prefix" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{5CB772C2-CF05-454F-BBBD-8EDEC112C696}" name="num_port_ledig" dataDxfId="0">
-      <calculatedColumnFormula>IF($A29=1,F29-G29-H29*$F$26-2,F29-G29-(1+H29)*$F$26-1)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{065F9F0A-8DB1-44A2-B7B3-97742E5CD0E1}" name="MONITORING ip">
-      <calculatedColumnFormula>LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{95B0B071-F602-4A16-BA0D-4B172283BAE9}" name="Tabell6214" displayName="Tabell6214" ref="A4:K9">
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{94861C51-5403-456D-87AF-7FC76DBA28A5}" name="vrf"/>
-    <tableColumn id="2" xr3:uid="{50243E8E-018E-40C1-A37D-ED67F4B092B0}" name="vlan"/>
-    <tableColumn id="3" xr3:uid="{A63B107D-5FA2-40D8-A99A-E280CFCC8C79}" name="interface"/>
-    <tableColumn id="4" xr3:uid="{A4267435-D295-44C3-B51E-0D1F4DD5C78B}" name="nett id">
-      <calculatedColumnFormula>10&amp;"."&amp;(B5+$A$2)&amp;"."&amp;0&amp;"."&amp;0</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="5" xr3:uid="{DC7B96FF-EAB7-4E6B-8DE8-85902CDECD19}" name="gateway">
-      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{1D8E9334-405A-4906-8238-47E036EC7609}" name="mask"/>
-    <tableColumn id="7" xr3:uid="{B5F525F7-1C0B-4D5D-BD37-F7614B933163}" name="address min">
-      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" xr3:uid="{BB245EF9-E497-4445-9E11-811371F6669C}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{8BE1DAE2-2DC3-4655-8CD3-ACB1B1D4A0F3}" name="antall-res" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{7934A4A2-4EDA-4DF0-9DAF-BA3DD0375EC2}" name="pri-afxx"/>
-    <tableColumn id="11" xr3:uid="{D8ADAB0C-E2D6-490F-A501-86D8C692367E}" name="pri-1-10"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{3B6A134F-5EA0-448A-B9C1-D15432398AB5}" name="Tabell7715" displayName="Tabell7715" ref="A11:C16">
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FA02FDEA-9585-4542-97E7-C1202764FFEC}" name="vrf"/>
-    <tableColumn id="3" xr3:uid="{840408ED-7E47-4F28-B0EB-9EDF05B3AEB2}" name="loopback"/>
-    <tableColumn id="4" xr3:uid="{FCE403FB-283B-4BF0-B99C-780D900D988D}" name="laddr">
-      <calculatedColumnFormula>$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(B12)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabell6" displayName="Tabell6" ref="A4:K9">
   <tableColumns count="11">
@@ -1581,7 +1087,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="33"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="pri-1-10"/>
   </tableColumns>
@@ -1611,7 +1117,7 @@
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="mask"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="63">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="32">
       <calculatedColumnFormula>$C$2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="destination"/>
@@ -1625,48 +1131,48 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A25:H26" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A25:H26" dataDxfId="31">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="61">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="30">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="59"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="span_mode" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{A8B916C7-04E3-4A58-909F-34F3F1BEB3E4}" name="erspan_destination" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="span_mode" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{A8B916C7-04E3-4A58-909F-34F3F1BEB3E4}" name="erspan_destination" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell1618242825" displayName="Tabell1618242825" ref="A28:L30" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell1618242825" displayName="Tabell1618242825" ref="A28:L29" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="53">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="22">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="51">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="20">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A29)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="50">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="19">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="49">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="18">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="48"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="43">
-      <calculatedColumnFormula>IF($A29=1,F29-G29-H29*$F$26-2-IF(OR($G$26="ERSPAN",$G$26="SPAN",$G$26="RSPAN"),1,0),F29-G29-(1+H29)*$F$26-1)</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="12">
+      <calculatedColumnFormula>IF($A29=1,F29-G29-H29*$F$26-2-IF(OR(UPPER($G$26)="SPAN", UPPER($G$26)="ERSPAN",UPPER($G$26)="RSPAN"),1,0),F29-G29-(1+H29)*$F$26-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{F45C6C35-68DB-43FE-9CBF-B6A2844A42CD}" name="MONITORING ip" dataDxfId="42">
+    <tableColumn id="12" xr3:uid="{F45C6C35-68DB-43FE-9CBF-B6A2844A42CD}" name="MONITORING ip" dataDxfId="11">
       <calculatedColumnFormula>LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1675,59 +1181,59 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:I2" dataDxfId="110">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:I2" dataDxfId="68">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="105"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="103"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="102">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="60">
       <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="dns_servers" dataDxfId="101"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="dns_servers" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A18:J23" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A18:J23" dataDxfId="58">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="98"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="97">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="55">
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="96"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="95">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="53">
       <calculatedColumnFormula>$C$2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="94"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="93"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="92"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="91"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="90"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A25:H26" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A25:H26" dataDxfId="47">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="88">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="46">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="86"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="etherchan_num" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="span_mode" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{BFD011F6-587B-466E-BAE0-BEEA0A83891E}" name="erspan_destination" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="etherchan_num" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="span_mode" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{BFD011F6-587B-466E-BAE0-BEEA0A83891E}" name="erspan_destination" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1928,7 +1434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1005"/>
+  <dimension ref="A1:L1004"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -2213,7 +1719,7 @@
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B9" s="9">
         <v>50</v>
@@ -2315,7 +1821,7 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="8">
         <v>50</v>
@@ -2476,10 +1982,10 @@
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C23" s="8" t="str">
         <f t="shared" ref="C23" si="12">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H23+$A$2)</f>
@@ -2536,7 +2042,7 @@
         <v>49</v>
       </c>
       <c r="H25" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="28.7" customHeight="1" x14ac:dyDescent="0.2">
@@ -2557,25 +2063,25 @@
         <v>12</v>
       </c>
       <c r="F26" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="H26" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="C28" s="15" t="s">
         <v>52</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>20</v>
@@ -2584,25 +2090,25 @@
         <v>21</v>
       </c>
       <c r="F28" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="I28" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>57</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>1</v>
       </c>
       <c r="K28" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2626,72 +2132,28 @@
         <v>255.255.0.0</v>
       </c>
       <c r="F29" s="8">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="G29" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="11">
-        <v>3</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>59</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I29" s="8"/>
       <c r="J29" s="2" t="s">
         <v>10</v>
       </c>
       <c r="K29" s="2">
         <f>IF($A29=1,F29-G29-H29*$F$26-2-IF(OR(UPPER($G$26)="SPAN", UPPER($G$26)="ERSPAN",UPPER($G$26)="RSPAN"),1,0),F29-G29-(1+H29)*$F$26-1)</f>
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="L29" t="str">
-        <f t="shared" ref="L29:L30" si="13">LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</f>
+        <f t="shared" ref="L29" si="13">LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</f>
         <v>10.51.0.2</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="17">
-        <v>2</v>
-      </c>
-      <c r="B30" s="17">
-        <v>10</v>
-      </c>
-      <c r="C30" s="17" t="str">
-        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A30)</f>
-        <v>10.11.0.3</v>
-      </c>
-      <c r="D30" s="17" t="str">
-        <f>$E$5</f>
-        <v>10.11.0.1</v>
-      </c>
-      <c r="E30" s="17" t="str">
-        <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F30" s="17">
-        <v>24</v>
-      </c>
-      <c r="G30" s="17">
-        <v>1</v>
-      </c>
-      <c r="H30" s="17">
-        <v>0</v>
-      </c>
-      <c r="I30" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="K30" s="2">
-        <f>IF($A30=1,F30-G30-H30*$F$26-2-IF(OR(UPPER($G$26)="SPAN",UPPER($G$26)="RSPAN"),1,0),F30-G30-(1+H30)*$F$26-1)</f>
-        <v>20</v>
-      </c>
-      <c r="L30" t="str">
-        <f t="shared" si="13"/>
-        <v>10.51.0.3</v>
-      </c>
-    </row>
+    <row r="30" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="31" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="32" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3666,14 +3128,13 @@
     <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1003" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1004" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1005" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I29:I30" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>IF(I29="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I29,"-"),"."))&lt;=K29)</formula1>
-    </dataValidation>
     <dataValidation type="list" sqref="G26" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"SPAN,RSPAN,ERSPAN"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I29" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>IF(I29="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I29,"-"),"."))&lt;=K29)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3962,7 +3423,7 @@
     </row>
     <row r="9" spans="1:11" s="14" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B9" s="9">
         <v>50</v>
@@ -4113,7 +3574,7 @@
     </row>
     <row r="16" spans="1:11" s="14" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="8">
         <v>50</v>
@@ -4281,35 +3742,35 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="18" t="str">
+      <c r="A23" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="16" t="str">
         <f t="shared" si="5"/>
         <v>172.16.0.52</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="18" t="str">
+      <c r="E23" s="16" t="str">
         <f t="shared" si="4"/>
         <v>2.2.2.0</v>
       </c>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18" t="s">
+      <c r="F23" s="16"/>
+      <c r="G23" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="16">
         <v>50</v>
       </c>
       <c r="I23" s="14" t="b">
         <f>'Site 1 (HUB)'!I23</f>
         <v>1</v>
       </c>
-      <c r="J23" s="19"/>
+      <c r="J23" s="17"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="25" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4335,7 +3796,7 @@
         <v>49</v>
       </c>
       <c r="H25" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4356,25 +3817,25 @@
         <v>12</v>
       </c>
       <c r="F26" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="H26" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="C28" s="15" t="s">
         <v>52</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>20</v>
@@ -4383,28 +3844,28 @@
         <v>21</v>
       </c>
       <c r="F28" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="I28" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>57</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>1</v>
       </c>
       <c r="K28" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L28" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <f>(ROW())-(ROW()-1)</f>
         <v>1</v>
@@ -4425,26 +3886,24 @@
         <v>255.255.0.0</v>
       </c>
       <c r="F29" s="8">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="G29" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="11">
         <v>0</v>
       </c>
-      <c r="I29" s="8" t="s">
-        <v>59</v>
-      </c>
+      <c r="I29" s="8"/>
       <c r="J29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K29" s="2">
-        <f>IF($A29=1,F29-G29-H29*$F$26-2,F29-G29-(1+H29)*$F$26-1)</f>
+      <c r="K29" s="2" cm="1">
+        <f t="array" ref="K29">[1]!Tabell161824282532[num_port_ledig]</f>
         <v>21</v>
       </c>
       <c r="L29" t="str">
-        <f>LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</f>
+        <f t="shared" ref="L29" si="6">LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</f>
         <v>10.52.0.2</v>
       </c>
     </row>
@@ -5419,7 +4878,7 @@
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I29" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I29" xr:uid="{D2AD5624-A156-47D7-A0C6-A47F59F949C5}">
       <formula1>IF(I29="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I29,"-"),"."))&lt;=K29)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="G26" xr:uid="{00000000-0002-0000-0100-000001000000}">
@@ -5436,799 +4895,4 @@
     <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L29"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="75.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="5" width="75.85546875" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="58.7109375" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="25.5703125" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="14">
-        <v>3</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="14" t="str">
-        <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</f>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="14" t="str">
-        <f>'Site 1 (HUB)'!H2</f>
-        <v>TACACS-KEY</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-    </row>
-    <row r="3" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-    </row>
-    <row r="4" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="9">
-        <v>10</v>
-      </c>
-      <c r="C5" s="8">
-        <v>0</v>
-      </c>
-      <c r="D5" s="8" t="str">
-        <f>10&amp;"."&amp;(B5+$A$2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.13.0.0</v>
-      </c>
-      <c r="E5" s="8" t="str">
-        <f>LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G9" si="0">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="H5" s="8" t="str">
-        <f>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</f>
-        <v>10.13.255.254</v>
-      </c>
-      <c r="I5" s="8">
-        <v>10</v>
-      </c>
-      <c r="J5" s="10">
-        <v>21</v>
-      </c>
-      <c r="K5" s="10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="9">
-        <v>20</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0</v>
-      </c>
-      <c r="D6" s="8" t="str">
-        <f t="shared" ref="D6:D9" si="1">10&amp;"."&amp;(B6+$A$2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.23.0.0</v>
-      </c>
-      <c r="E6" s="8" t="str">
-        <f t="shared" ref="E6:E9" si="2">LEFT(D6,LEN(D6)-1)&amp;"1"</f>
-        <v>10.23.0.1</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>10.23.0.1</v>
-      </c>
-      <c r="H6" s="8" t="str">
-        <f>LEFT(D6,FIND(".",D6,FIND(".",D6)+1)-1)&amp;".255.254"</f>
-        <v>10.23.255.254</v>
-      </c>
-      <c r="I6" s="8">
-        <v>10</v>
-      </c>
-      <c r="J6" s="10">
-        <v>11</v>
-      </c>
-      <c r="K6" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="9">
-        <v>30</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>10.33.0.0</v>
-      </c>
-      <c r="E7" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>10.33.0.1</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>10.33.0.1</v>
-      </c>
-      <c r="H7" s="8" t="str">
-        <f>LEFT(D7,FIND(".",D7,FIND(".",D7)+1)-1)&amp;".255.254"</f>
-        <v>10.33.255.254</v>
-      </c>
-      <c r="I7" s="8">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>42</v>
-      </c>
-      <c r="K7">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="9">
-        <v>40</v>
-      </c>
-      <c r="C8" s="8">
-        <v>0</v>
-      </c>
-      <c r="D8" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>10.43.0.0</v>
-      </c>
-      <c r="E8" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>10.43.0.1</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>10.43.0.1</v>
-      </c>
-      <c r="H8" s="8" t="str">
-        <f>LEFT(D8,FIND(".",D8,FIND(".",D8)+1)-1)&amp;".255.254"</f>
-        <v>10.43.255.254</v>
-      </c>
-      <c r="I8" s="8">
-        <v>10</v>
-      </c>
-      <c r="J8">
-        <v>41</v>
-      </c>
-      <c r="K8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="9">
-        <v>50</v>
-      </c>
-      <c r="C9" s="8">
-        <v>0</v>
-      </c>
-      <c r="D9" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>10.53.0.0</v>
-      </c>
-      <c r="E9" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>10.53.0.1</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>10.53.0.1</v>
-      </c>
-      <c r="H9" s="8" t="str">
-        <f>LEFT(D9,FIND(".",D9,FIND(".",D9)+1)-1)&amp;".0.254"</f>
-        <v>10.53.0.254</v>
-      </c>
-      <c r="I9" s="8">
-        <v>10</v>
-      </c>
-      <c r="J9">
-        <v>43</v>
-      </c>
-      <c r="K9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="8">
-        <v>10</v>
-      </c>
-      <c r="C12" s="8" t="str">
-        <f>$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(B12)</f>
-        <v>3.3.3.10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="8">
-        <v>20</v>
-      </c>
-      <c r="C13" s="8" t="str">
-        <f t="shared" ref="C13:C16" si="3">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(B13)</f>
-        <v>3.3.3.20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="8">
-        <v>30</v>
-      </c>
-      <c r="C14" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>3.3.3.30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="8">
-        <v>40</v>
-      </c>
-      <c r="C15" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>3.3.3.40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="8">
-        <v>50</v>
-      </c>
-      <c r="C16" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>3.3.3.50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-    </row>
-    <row r="18" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J18" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="14"/>
-    </row>
-    <row r="19" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="14" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
-        <v>172.16.0.13</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E19" s="14" t="str">
-        <f t="shared" ref="E19:E23" si="4">$C$2</f>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H19" s="14">
-        <v>10</v>
-      </c>
-      <c r="I19" s="14">
-        <f t="array" ref="I19">'Site 1 (HUB)'!I19</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-    </row>
-    <row r="20" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="14" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H20+$A$2)</f>
-        <v>172.16.0.23</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="14" t="str">
-        <f t="shared" si="4"/>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" s="14">
-        <v>20</v>
-      </c>
-      <c r="I20" s="14" cm="1">
-        <f t="array" ref="I20">'Site 1 (HUB)'!I20</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-    </row>
-    <row r="21" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="14" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H21+$A$2)</f>
-        <v>172.16.0.33</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E21" s="14" t="str">
-        <f t="shared" si="4"/>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H21" s="14">
-        <v>30</v>
-      </c>
-      <c r="I21" s="14" t="b">
-        <f>'Site 1 (HUB)'!I21</f>
-        <v>1</v>
-      </c>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-    </row>
-    <row r="22" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="14" t="str">
-        <f t="shared" ref="C22:C23" si="5">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H22+$A$2)</f>
-        <v>172.16.0.43</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E22" s="14" t="str">
-        <f t="shared" si="4"/>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H22" s="14">
-        <v>40</v>
-      </c>
-      <c r="I22" s="14" t="b">
-        <f>'Site 1 (HUB)'!I22</f>
-        <v>1</v>
-      </c>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-    </row>
-    <row r="23" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v>172.16.0.53</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="18" t="str">
-        <f t="shared" si="4"/>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="H23" s="18">
-        <v>50</v>
-      </c>
-      <c r="I23" s="14" t="b">
-        <f>'Site 1 (HUB)'!I23</f>
-        <v>1</v>
-      </c>
-      <c r="J23" s="19"/>
-      <c r="K23" s="14"/>
-    </row>
-    <row r="24" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="14"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-    </row>
-    <row r="25" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H25" t="s">
-        <v>60</v>
-      </c>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-    </row>
-    <row r="26" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="14">
-        <f>A2</f>
-        <v>3</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="14">
-        <v>2</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-    </row>
-    <row r="27" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-    </row>
-    <row r="28" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="H28" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="L28" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
-        <f>(ROW())-(ROW()-1)</f>
-        <v>1</v>
-      </c>
-      <c r="B29" s="8">
-        <v>10</v>
-      </c>
-      <c r="C29" s="8" t="str">
-        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A29)</f>
-        <v>10.13.0.2</v>
-      </c>
-      <c r="D29" s="8" t="str">
-        <f>$E$5</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="E29" s="8" t="str">
-        <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F29" s="8">
-        <v>24</v>
-      </c>
-      <c r="G29" s="8">
-        <v>1</v>
-      </c>
-      <c r="H29" s="11">
-        <v>0</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K29" s="2">
-        <f>IF($A29=1,F29-G29-H29*$F$26-2,F29-G29-(1+H29)*$F$26-1)</f>
-        <v>21</v>
-      </c>
-      <c r="L29" t="str">
-        <f>LEFT($G$9,LEN($G$9)-1)&amp;(RIGHT($G$9,1)+A29)</f>
-        <v>10.53.0.2</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I29" xr:uid="{7287270F-FA36-42B0-936E-CB6AE119A013}">
-      <formula1>IF(I29="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I29,"-"),"."))&lt;=K29)</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="G26" xr:uid="{96B8245A-DA04-4B17-A070-977D41BECEDD}">
-      <formula1>"SPAN,RSPAN,ERSPAN"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="6">
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
-    <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>